<commit_message>
Create one site resource per email, with computed city-based names
Each User Emails entry on a row now creates its own site resource
(a row with 3 emails creates 3 resources) instead of one shared
multi-user resource per row, so access and naming are per-user.
Resource names are computed as <city>-<username>-<vlan>[-<z>] from
the Name (city) column, the email's local part, and the Destination
IP's octets, rather than typed in directly.

Unresolved emails and emailless rows are skipped locally (no API
call) and reported as FAIL rows instead of silently dropped or
grouped into a shared resource. Results report reshaped to one row
per attempted resource/skipped email.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pangolin_private_resources_template.xlsx
+++ b/pangolin_private_resources_template.xlsx
@@ -1,22 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyData\Τζιρτζιλάκης\ΜΨΔ\Pangolin\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F6EE67-AFC7-45CB-BCD9-F69138E2A939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="2745" windowWidth="38700" windowHeight="15285" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Οδηγίες" sheetId="1" r:id="rId1"/>
-    <sheet name="Requests" sheetId="2" r:id="rId2"/>
+    <sheet name="Οδηγίες" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Requests" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -26,152 +21,106 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
-  <si>
-    <t>Αίτημα Δημιουργίας Ιδιωτικού Πόρου Pangolin — Οδηγίες</t>
-  </si>
-  <si>
-    <t>Συμπληρώστε μία γραμμή ανά ιδιωτικό πόρο στο φύλλο "Requests" και επιστρέψτε το αρχείο.</t>
-  </si>
-  <si>
-    <t>Μην αλλάζετε τις επικεφαλίδες των στηλών και μην προσθέτετε νέες στήλες.</t>
-  </si>
-  <si>
-    <t>Στήλη: Name</t>
-  </si>
-  <si>
-    <t>Συμπληρώνεται αργότερα από τη Μονάδα Ψηφιακής Διακυβέρνησης</t>
-  </si>
-  <si>
-    <t>Στήλη: Destination (IP or CIDR)</t>
-  </si>
-  <si>
-    <t>Υποχρεωτικό. Είτε μία μεμονωμένη IP διεύθυνση host (π.χ. 10.23.25.11) είτε ένα εύρος CIDR για ολόκληρο υποδίκτυο (π.χ. 10.23.25.0/24). Μία μεμονωμένη IP αντιμετωπίζεται ως πόρος τύπου "host", ενώ ένα CIDR αντιμετωπίζεται ως πόρος τύπου "δικτύου" (network/subnet).</t>
-  </si>
-  <si>
-    <t>Στήλη: Alias</t>
-  </si>
-  <si>
-    <t>Προαιρετικό. Εναλλακτικό/φιλικό όνομα (hostname) για τον πόρο, π.χ. rdp-server-a.internal. Χρησιμοποιείται μόνο αν θέλετε να προσπελαύνετε τον πόρο μέσω ονόματος αντί IP.  Δεν ισχύει στην περίπτωση εύρους CIDR. Αν δεν χρειάζεστε κάτι τέτοιο, αφήστε το κενό.</t>
-  </si>
-  <si>
-    <t>Στήλη: User Emails</t>
-  </si>
-  <si>
-    <t>Στήλη: Notes</t>
-  </si>
-  <si>
-    <t>Προαιρετικό. Οποιαδήποτε άλλη σχετική πληροφορία για το αίτημα.</t>
-  </si>
-  <si>
-    <t>Παραδείγματα</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Destination</t>
-  </si>
-  <si>
-    <t>Alias</t>
-  </si>
-  <si>
-    <t>User Emails</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>10.23.25.11</t>
-  </si>
-  <si>
-    <t>user1@uop.gr</t>
-  </si>
-  <si>
-    <t>10.23.30.0/24</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>user1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">@uop.gr, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>user2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <charset val="1"/>
-      </rPr>
-      <t>@uop.gr</t>
-    </r>
-  </si>
-  <si>
-    <t>Ολόκληρο υποδίκτυο</t>
-  </si>
-  <si>
-    <t>10.23.25.14</t>
-  </si>
-  <si>
-    <t>app14.internal</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>user1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <charset val="1"/>
-      </rPr>
-      <t>@uop.gr</t>
-    </r>
-  </si>
-  <si>
-    <t>Destination (IP or CIDR)</t>
-  </si>
-  <si>
-    <t>Λίστα email (χωρισμένα με κόμμα) των χρηστών που θα έχουν πρόσβαση σε αυτόν τον πόρο, π.χ. user1@uop.gr, user2@uop.gr. Πρόσβαση θα έχουν ΜΟΝΟ αυτοί οι χρήστες — όχι πρόσβαση βάσει ρόλου (role).</t>
-  </si>
-  <si>
-    <t>Operation System</t>
-  </si>
-  <si>
-    <t>Name (Συμπληρώνεται από τη ΜΨΔ)</t>
-  </si>
-  <si>
-    <t>Στήλη: Operation System</t>
-  </si>
-  <si>
-    <t>Συμπληρώνετε Linux ή Windows</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+  <si>
+    <t xml:space="preserve">Αίτημα Δημιουργίας Ιδιωτικού Πόρου Pangolin — Οδηγίες</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Συμπληρώστε μία γραμμή ανά ιδιωτικό πόρο στο φύλλο "Requests" και επιστρέψτε το αρχείο.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Μην αλλάζετε τις επικεφαλίδες των στηλών και μην προσθέτετε νέες στήλες.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Συμπληρώνεται αργότερα από τη Μονάδα Ψηφιακής Διακυβέρνησης με την πόλη/τοποθεσία του πόρου (π.χ. "Πάτρα") — δεν συμπληρώνεται από τον αιτούντα. Χρησιμοποιείται ως το πρώτο τμήμα του τελικού ονόματος του πόρου (βλ. στήλη User Emails).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: Operation System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Συμπληρώνετε Linux ή Windows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: Destination (IP or CIDR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Υποχρεωτικό. Είτε μία μεμονωμένη IP διεύθυνση host (π.χ. 10.23.25.11) είτε ένα εύρος CIDR για ολόκληρο υποδίκτυο (π.χ. 10.23.25.0/24). Μία μεμονωμένη IP αντιμετωπίζεται ως πόρος τύπου "host", ενώ ένα CIDR αντιμετωπίζεται ως πόρος τύπου "δικτύου" (network/subnet).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: Alias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Προαιρετικό. Εναλλακτικό/φιλικό όνομα (hostname) για τον πόρο, π.χ. rdp-server-a.internal. Χρησιμοποιείται μόνο αν θέλετε να προσπελαύνετε τον πόρο μέσω ονόματος αντί IP.  Δεν ισχύει στην περίπτωση εύρους CIDR. Αν δεν χρειάζεστε κάτι τέτοιο, αφήστε το κενό.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: User Emails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Λίστα email (χωρισμένα με κόμμα) των χρηστών που θα έχουν πρόσβαση σε αυτόν τον πόρο, π.χ. user1@uop.gr, user2@uop.gr. Κάθε email δημιουργεί τον ΔΙΚΟ ΤΟΥ ξεχωριστό πόρο (π.χ. 2 email = 2 πόροι), ώστε η πρόσβαση να δίνεται ξεχωριστά ανά χρήστη — όχι πρόσβαση βάσει ρόλου (role). Το όνομα κάθε πόρου παράγεται αυτόματα ως "&lt;πόλη&gt;-&lt;username&gt;-&lt;vlan&gt;-&lt;z&gt;" (π.χ. ktsouvalis@uop.gr στο 10.23.2.50, πόλη "Πάτρα" -&gt; patra-ktsouvalis-2302-50).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Στήλη: Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Προαιρετικό. Οποιαδήποτε άλλη σχετική πληροφορία για το αίτημα.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Παραδείγματα</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operation System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User Emails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.23.25.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user1@uop.gr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.23.30.0/24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user1@uop.gr, user2@uop.gr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ολόκληρο υποδίκτυο</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.23.25.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name (Συμπληρώνεται από τη ΜΨΔ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destination (IP or CIDR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alias</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,36 +131,52 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -236,14 +201,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -259,26 +224,73 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Κανονικό" xfId="0" builtinId="0"/>
+  <cellStyles count="6">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -337,63 +349,47 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -401,12 +397,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -435,7 +431,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -456,7 +452,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -507,7 +503,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -525,208 +521,209 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" customWidth="1"/>
-    <col min="6" max="8" width="22" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="27.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="4" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="4" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="4" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2" t="s">
+      <c r="C25" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2" t="s">
+      <c r="D25" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2" t="s">
+      <c r="E25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="2"/>
-      <c r="E27" s="5" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="2" t="s">
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="5"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="3"/>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F61"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" customFormat="false" ht="44.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="E1" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -734,7 +731,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -742,7 +739,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -750,7 +747,7 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -758,7 +755,7 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -766,7 +763,7 @@
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -774,7 +771,7 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -782,7 +779,7 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -790,7 +787,7 @@
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -798,7 +795,7 @@
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -806,7 +803,7 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -814,7 +811,7 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -822,7 +819,7 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -830,7 +827,7 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -838,7 +835,7 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -846,7 +843,7 @@
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -854,7 +851,7 @@
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -862,7 +859,7 @@
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -870,7 +867,7 @@
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -878,7 +875,7 @@
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -886,7 +883,7 @@
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -894,7 +891,7 @@
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -902,7 +899,7 @@
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -910,7 +907,7 @@
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -918,7 +915,7 @@
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -926,7 +923,7 @@
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -934,7 +931,7 @@
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -942,7 +939,7 @@
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -950,7 +947,7 @@
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -958,7 +955,7 @@
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -966,7 +963,7 @@
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -974,7 +971,7 @@
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7"/>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -982,7 +979,7 @@
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -990,7 +987,7 @@
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
@@ -998,7 +995,7 @@
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
@@ -1006,7 +1003,7 @@
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
@@ -1014,7 +1011,7 @@
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -1022,7 +1019,7 @@
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
@@ -1030,7 +1027,7 @@
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
@@ -1038,7 +1035,7 @@
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
@@ -1046,7 +1043,7 @@
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
@@ -1054,7 +1051,7 @@
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
@@ -1062,7 +1059,7 @@
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
@@ -1070,7 +1067,7 @@
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
@@ -1078,7 +1075,7 @@
       <c r="E45" s="7"/>
       <c r="F45" s="7"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
@@ -1086,7 +1083,7 @@
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
@@ -1094,7 +1091,7 @@
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
@@ -1102,7 +1099,7 @@
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
@@ -1110,7 +1107,7 @@
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7"/>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
@@ -1118,7 +1115,7 @@
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
@@ -1126,7 +1123,7 @@
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7"/>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
@@ -1134,7 +1131,7 @@
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7"/>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
@@ -1142,7 +1139,7 @@
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
@@ -1150,7 +1147,7 @@
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7"/>
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
@@ -1158,7 +1155,7 @@
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
@@ -1166,7 +1163,7 @@
       <c r="E56" s="7"/>
       <c r="F56" s="7"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7"/>
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
@@ -1174,7 +1171,7 @@
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
@@ -1182,7 +1179,7 @@
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
@@ -1190,7 +1187,7 @@
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
@@ -1198,7 +1195,7 @@
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7"/>
       <c r="B61" s="7"/>
       <c r="C61" s="7"/>
@@ -1207,7 +1204,12 @@
       <c r="F61" s="7"/>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>